<commit_message>
Final Sync V68: admin/Reporte_Comisiones_por_Vendedor_OFICIAL.xlsx
</commit_message>
<xml_diff>
--- a/admin/Reporte_Comisiones_por_Vendedor_OFICIAL.xlsx
+++ b/admin/Reporte_Comisiones_por_Vendedor_OFICIAL.xlsx
@@ -539,14 +539,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="29" customWidth="1" min="9" max="9"/>
@@ -562,7 +562,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Regla Oficial: Se liquida comisión en pedidos ENTREGADOS (status='recibido'). Devoluciones = $0. En despacho = Pendiente.</t>
+          <t>Regla Negocio: Solo se liquida comisión en pedidos RECIBIDOS con DINERO CONFIRMADO.</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Ventas Liquidadas (Entregadas)</t>
+          <t>Ventas Liquidadas (Recibidas+$)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Ventas Pendientes (En Despacho)</t>
+          <t>Ventas Pendientes (Despacho)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -720,16 +720,16 @@
         <v>5470000</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>215000</v>
+        <v>190000</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>55000</v>
+        <v>80000</v>
       </c>
       <c r="H8" s="5" t="n">
         <v>0</v>
@@ -751,13 +751,13 @@
         <v>31475441</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" s="8" t="n">
         <v>0</v>
@@ -782,13 +782,13 @@
         <v>151412000</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="E10" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>0</v>
@@ -844,13 +844,13 @@
         <v>204844002</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="E12" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>0</v>
@@ -912,7 +912,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N280"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -924,8 +924,8 @@
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="29" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="35" customWidth="1" min="12" max="12"/>
     <col width="37" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
   </cols>
@@ -998,7 +998,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Entregado / Confirmado</t>
+          <t>Dinero Confirmado</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -1728,18 +1728,18 @@
       </c>
       <c r="K15" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L15" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M15" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L15" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4632,18 +4632,18 @@
       </c>
       <c r="K59" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L59" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M59" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N59" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L59" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M59" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12486,18 +12486,18 @@
       </c>
       <c r="K178" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L178" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M178" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N178" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L178" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M178" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N178" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -17304,18 +17304,18 @@
       </c>
       <c r="K251" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L251" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M251" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N251" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L251" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M251" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N251" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -17436,12 +17436,12 @@
       </c>
       <c r="K253" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L253" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (Sin Despachar)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M253" s="16" t="n">
@@ -19208,7 +19208,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N633"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -19220,8 +19220,8 @@
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="35" customWidth="1" min="12" max="12"/>
     <col width="37" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
   </cols>
@@ -19294,7 +19294,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Entregado / Confirmado</t>
+          <t>Dinero Confirmado</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -19369,7 +19369,7 @@
       </c>
       <c r="L5" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M5" s="16" t="n">
@@ -21217,7 +21217,7 @@
       </c>
       <c r="L33" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M33" s="16" t="n">
@@ -22141,7 +22141,7 @@
       </c>
       <c r="L47" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M47" s="16" t="n">
@@ -22207,7 +22207,7 @@
       </c>
       <c r="L48" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M48" s="16" t="n">
@@ -23065,7 +23065,7 @@
       </c>
       <c r="L61" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M61" s="16" t="n">
@@ -23923,7 +23923,7 @@
       </c>
       <c r="L74" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M74" s="16" t="n">
@@ -23989,7 +23989,7 @@
       </c>
       <c r="L75" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M75" s="16" t="n">
@@ -24781,7 +24781,7 @@
       </c>
       <c r="L87" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M87" s="16" t="n">
@@ -24847,7 +24847,7 @@
       </c>
       <c r="L88" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M88" s="16" t="n">
@@ -24913,7 +24913,7 @@
       </c>
       <c r="L89" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M89" s="16" t="n">
@@ -25903,7 +25903,7 @@
       </c>
       <c r="L104" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M104" s="16" t="n">
@@ -25969,7 +25969,7 @@
       </c>
       <c r="L105" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M105" s="16" t="n">
@@ -26035,7 +26035,7 @@
       </c>
       <c r="L106" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M106" s="16" t="n">
@@ -26101,7 +26101,7 @@
       </c>
       <c r="L107" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M107" s="16" t="n">
@@ -26167,7 +26167,7 @@
       </c>
       <c r="L108" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M108" s="16" t="n">
@@ -26233,7 +26233,7 @@
       </c>
       <c r="L109" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M109" s="16" t="n">
@@ -26827,7 +26827,7 @@
       </c>
       <c r="L118" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M118" s="16" t="n">
@@ -26893,7 +26893,7 @@
       </c>
       <c r="L119" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M119" s="16" t="n">
@@ -26959,7 +26959,7 @@
       </c>
       <c r="L120" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M120" s="16" t="n">
@@ -27025,7 +27025,7 @@
       </c>
       <c r="L121" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M121" s="16" t="n">
@@ -27091,7 +27091,7 @@
       </c>
       <c r="L122" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M122" s="16" t="n">
@@ -27157,7 +27157,7 @@
       </c>
       <c r="L123" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M123" s="16" t="n">
@@ -27289,7 +27289,7 @@
       </c>
       <c r="L125" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M125" s="16" t="n">
@@ -27355,7 +27355,7 @@
       </c>
       <c r="L126" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M126" s="16" t="n">
@@ -27883,7 +27883,7 @@
       </c>
       <c r="L134" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M134" s="16" t="n">
@@ -27949,7 +27949,7 @@
       </c>
       <c r="L135" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M135" s="16" t="n">
@@ -28015,7 +28015,7 @@
       </c>
       <c r="L136" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M136" s="16" t="n">
@@ -28081,7 +28081,7 @@
       </c>
       <c r="L137" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M137" s="16" t="n">
@@ -28147,7 +28147,7 @@
       </c>
       <c r="L138" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M138" s="16" t="n">
@@ -28213,7 +28213,7 @@
       </c>
       <c r="L139" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M139" s="16" t="n">
@@ -28279,7 +28279,7 @@
       </c>
       <c r="L140" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M140" s="16" t="n">
@@ -28345,7 +28345,7 @@
       </c>
       <c r="L141" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M141" s="16" t="n">
@@ -28411,7 +28411,7 @@
       </c>
       <c r="L142" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M142" s="16" t="n">
@@ -28477,7 +28477,7 @@
       </c>
       <c r="L143" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M143" s="16" t="n">
@@ -28543,7 +28543,7 @@
       </c>
       <c r="L144" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M144" s="16" t="n">
@@ -28609,7 +28609,7 @@
       </c>
       <c r="L145" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M145" s="16" t="n">
@@ -28675,7 +28675,7 @@
       </c>
       <c r="L146" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M146" s="16" t="n">
@@ -28741,7 +28741,7 @@
       </c>
       <c r="L147" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M147" s="16" t="n">
@@ -28807,7 +28807,7 @@
       </c>
       <c r="L148" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M148" s="16" t="n">
@@ -28873,7 +28873,7 @@
       </c>
       <c r="L149" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M149" s="16" t="n">
@@ -28939,7 +28939,7 @@
       </c>
       <c r="L150" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M150" s="16" t="n">
@@ -29005,7 +29005,7 @@
       </c>
       <c r="L151" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M151" s="16" t="n">
@@ -29071,7 +29071,7 @@
       </c>
       <c r="L152" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M152" s="16" t="n">
@@ -29533,7 +29533,7 @@
       </c>
       <c r="L159" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M159" s="16" t="n">
@@ -29599,7 +29599,7 @@
       </c>
       <c r="L160" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M160" s="16" t="n">
@@ -30188,19 +30188,19 @@
       </c>
       <c r="K169" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L169" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M169" s="21" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L169" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M169" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N169" s="19" t="n">
         <v>25000</v>
-      </c>
-      <c r="N169" s="16" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="170">
@@ -30518,18 +30518,18 @@
       </c>
       <c r="K174" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L174" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M174" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N174" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L174" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M174" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N174" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -31310,18 +31310,18 @@
       </c>
       <c r="K186" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L186" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M186" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N186" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L186" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M186" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N186" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -31376,18 +31376,18 @@
       </c>
       <c r="K187" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L187" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M187" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N187" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L187" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M187" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N187" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -31970,18 +31970,18 @@
       </c>
       <c r="K196" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L196" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M196" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N196" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L196" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M196" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N196" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -34610,18 +34610,18 @@
       </c>
       <c r="K236" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L236" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M236" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N236" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L236" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M236" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N236" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -34676,18 +34676,18 @@
       </c>
       <c r="K237" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L237" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M237" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N237" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L237" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M237" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N237" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -34742,18 +34742,18 @@
       </c>
       <c r="K238" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L238" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M238" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N238" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L238" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M238" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N238" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -34808,18 +34808,18 @@
       </c>
       <c r="K239" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L239" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M239" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N239" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L239" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M239" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N239" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -34874,18 +34874,18 @@
       </c>
       <c r="K240" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L240" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M240" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N240" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L240" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M240" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N240" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -41342,18 +41342,18 @@
       </c>
       <c r="K338" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L338" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M338" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N338" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L338" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M338" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N338" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -52298,18 +52298,18 @@
       </c>
       <c r="K504" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L504" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M504" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N504" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L504" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M504" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N504" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -52364,18 +52364,18 @@
       </c>
       <c r="K505" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L505" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M505" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N505" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L505" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M505" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N505" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -58766,18 +58766,18 @@
       </c>
       <c r="K602" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L602" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M602" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N602" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L602" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M602" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N602" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -58898,12 +58898,12 @@
       </c>
       <c r="K604" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L604" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (Sin Despachar)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M604" s="16" t="n">
@@ -60802,7 +60802,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N143"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -60814,8 +60814,8 @@
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="35" customWidth="1" min="12" max="12"/>
     <col width="37" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
   </cols>
@@ -60888,7 +60888,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Entregado / Confirmado</t>
+          <t>Dinero Confirmado</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -62019,7 +62019,7 @@
       </c>
       <c r="L21" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M21" s="16" t="n">
@@ -62745,7 +62745,7 @@
       </c>
       <c r="L32" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M32" s="16" t="n">
@@ -63339,7 +63339,7 @@
       </c>
       <c r="L41" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M41" s="16" t="n">
@@ -64131,7 +64131,7 @@
       </c>
       <c r="L53" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M53" s="16" t="n">
@@ -64197,7 +64197,7 @@
       </c>
       <c r="L54" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M54" s="16" t="n">
@@ -64923,7 +64923,7 @@
       </c>
       <c r="L65" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M65" s="16" t="n">
@@ -64989,7 +64989,7 @@
       </c>
       <c r="L66" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M66" s="16" t="n">
@@ -65847,7 +65847,7 @@
       </c>
       <c r="L79" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M79" s="16" t="n">
@@ -65913,7 +65913,7 @@
       </c>
       <c r="L80" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M80" s="16" t="n">
@@ -65979,7 +65979,7 @@
       </c>
       <c r="L81" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M81" s="16" t="n">
@@ -66045,7 +66045,7 @@
       </c>
       <c r="L82" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M82" s="16" t="n">
@@ -66111,7 +66111,7 @@
       </c>
       <c r="L83" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M83" s="16" t="n">
@@ -66177,7 +66177,7 @@
       </c>
       <c r="L84" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M84" s="16" t="n">
@@ -66771,7 +66771,7 @@
       </c>
       <c r="L93" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M93" s="16" t="n">
@@ -66837,7 +66837,7 @@
       </c>
       <c r="L94" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M94" s="16" t="n">
@@ -66903,7 +66903,7 @@
       </c>
       <c r="L95" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M95" s="16" t="n">
@@ -66969,7 +66969,7 @@
       </c>
       <c r="L96" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M96" s="16" t="n">
@@ -67035,7 +67035,7 @@
       </c>
       <c r="L97" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M97" s="16" t="n">
@@ -67167,7 +67167,7 @@
       </c>
       <c r="L99" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M99" s="16" t="n">
@@ -67233,7 +67233,7 @@
       </c>
       <c r="L100" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M100" s="16" t="n">
@@ -67761,7 +67761,7 @@
       </c>
       <c r="L108" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M108" s="16" t="n">
@@ -67827,7 +67827,7 @@
       </c>
       <c r="L109" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M109" s="16" t="n">
@@ -67893,7 +67893,7 @@
       </c>
       <c r="L110" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M110" s="16" t="n">
@@ -67959,7 +67959,7 @@
       </c>
       <c r="L111" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M111" s="16" t="n">
@@ -68025,7 +68025,7 @@
       </c>
       <c r="L112" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M112" s="16" t="n">
@@ -68091,7 +68091,7 @@
       </c>
       <c r="L113" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M113" s="16" t="n">
@@ -68157,7 +68157,7 @@
       </c>
       <c r="L114" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M114" s="16" t="n">
@@ -68223,7 +68223,7 @@
       </c>
       <c r="L115" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M115" s="16" t="n">
@@ -68289,7 +68289,7 @@
       </c>
       <c r="L116" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M116" s="16" t="n">
@@ -68355,7 +68355,7 @@
       </c>
       <c r="L117" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M117" s="16" t="n">
@@ -68421,7 +68421,7 @@
       </c>
       <c r="L118" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M118" s="16" t="n">
@@ -68487,7 +68487,7 @@
       </c>
       <c r="L119" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M119" s="16" t="n">
@@ -68553,7 +68553,7 @@
       </c>
       <c r="L120" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M120" s="16" t="n">
@@ -68619,7 +68619,7 @@
       </c>
       <c r="L121" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M121" s="16" t="n">
@@ -68685,7 +68685,7 @@
       </c>
       <c r="L122" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M122" s="16" t="n">
@@ -68751,7 +68751,7 @@
       </c>
       <c r="L123" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M123" s="16" t="n">
@@ -68817,7 +68817,7 @@
       </c>
       <c r="L124" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M124" s="16" t="n">
@@ -68883,7 +68883,7 @@
       </c>
       <c r="L125" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M125" s="16" t="n">
@@ -68949,7 +68949,7 @@
       </c>
       <c r="L126" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M126" s="16" t="n">
@@ -69411,7 +69411,7 @@
       </c>
       <c r="L133" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M133" s="16" t="n">
@@ -69477,7 +69477,7 @@
       </c>
       <c r="L134" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M134" s="16" t="n">
@@ -70056,7 +70056,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -70068,7 +70068,7 @@
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
     <col width="28" customWidth="1" min="12" max="12"/>
     <col width="37" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
@@ -70142,7 +70142,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Entregado / Confirmado</t>
+          <t>Dinero Confirmado</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -70334,7 +70334,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -70346,7 +70346,7 @@
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
     <col width="28" customWidth="1" min="12" max="12"/>
     <col width="37" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
@@ -70420,7 +70420,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Entregado / Confirmado</t>
+          <t>Dinero Confirmado</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -71008,7 +71008,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -71020,8 +71020,8 @@
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="35" customWidth="1" min="12" max="12"/>
     <col width="37" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
   </cols>
@@ -71094,7 +71094,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Entregado / Confirmado</t>
+          <t>Dinero Confirmado</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -71499,7 +71499,7 @@
       </c>
       <c r="L10" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M10" s="16" t="n">
@@ -71829,7 +71829,7 @@
       </c>
       <c r="L15" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M15" s="16" t="n">
@@ -72027,7 +72027,7 @@
       </c>
       <c r="L18" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M18" s="16" t="n">
@@ -72154,19 +72154,19 @@
       </c>
       <c r="K20" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L20" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M20" s="21" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L20" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="19" t="n">
         <v>25000</v>
-      </c>
-      <c r="N20" s="16" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -72210,7 +72210,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -72222,8 +72222,8 @@
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="35" customWidth="1" min="12" max="12"/>
     <col width="37" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
   </cols>
@@ -72296,7 +72296,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Entregado / Confirmado</t>
+          <t>Dinero Confirmado</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -72498,18 +72498,18 @@
       </c>
       <c r="K7" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L7" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M7" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L7" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M7" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -73016,7 +73016,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N181"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -73028,8 +73028,8 @@
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="35" customWidth="1" min="12" max="12"/>
     <col width="37" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
   </cols>
@@ -73102,7 +73102,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Entregado / Confirmado</t>
+          <t>Dinero Confirmado</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -73436,18 +73436,18 @@
       </c>
       <c r="K9" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L9" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M9" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L9" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M9" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -73502,18 +73502,18 @@
       </c>
       <c r="K10" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L10" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M10" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -74096,18 +74096,18 @@
       </c>
       <c r="K19" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L19" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L19" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -76076,18 +76076,18 @@
       </c>
       <c r="K49" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L49" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M49" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N49" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L49" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M49" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N49" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -76142,18 +76142,18 @@
       </c>
       <c r="K50" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L50" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M50" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N50" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L50" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M50" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -76208,18 +76208,18 @@
       </c>
       <c r="K51" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L51" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M51" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N51" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L51" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M51" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -76274,18 +76274,18 @@
       </c>
       <c r="K52" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L52" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M52" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N52" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L52" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M52" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N52" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -83006,18 +83006,18 @@
       </c>
       <c r="K154" s="17" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L154" s="20" t="inlineStr">
-        <is>
-          <t>LIQUIDABLE (A Pagar Hoy)</t>
-        </is>
-      </c>
-      <c r="M154" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N154" s="16" t="n">
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L154" s="18" t="inlineStr">
+        <is>
+          <t>PENDIENTE (Dinero no ingresado)</t>
+        </is>
+      </c>
+      <c r="M154" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N154" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -84778,7 +84778,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -84790,8 +84790,8 @@
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="35" customWidth="1" min="12" max="12"/>
     <col width="37" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
   </cols>
@@ -84864,7 +84864,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Entregado / Confirmado</t>
+          <t>Dinero Confirmado</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -84939,7 +84939,7 @@
       </c>
       <c r="L5" s="18" t="inlineStr">
         <is>
-          <t>PENDIENTE (En Despacho / Tránsito)</t>
+          <t>PENDIENTE (Dinero no ingresado)</t>
         </is>
       </c>
       <c r="M5" s="16" t="n">

</xml_diff>